<commit_message>
Twincat update: 12.02 (15:03)
</commit_message>
<xml_diff>
--- a/Twincat/Parameters.xlsx
+++ b/Twincat/Parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kimro\Documents\Bachelor\Twincat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3070D0D-16B0-4248-80BE-6B96FA0B6D12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689332FD-F6D4-4377-BDE9-85228FBC28F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75D9AD79-BFC7-4289-9BE2-FD8EA15511B0}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>FB_ValveOutput_NC</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
   <si>
     <t>nOffset</t>
   </si>
@@ -66,6 +63,114 @@
   </si>
   <si>
     <t>Min value valve?</t>
+  </si>
+  <si>
+    <t>FB_Running</t>
+  </si>
+  <si>
+    <t>FB_ControllerMode</t>
+  </si>
+  <si>
+    <t>PRG_ControllerMode</t>
+  </si>
+  <si>
+    <t>P_Modes</t>
+  </si>
+  <si>
+    <t>FB_ValveOutput</t>
+  </si>
+  <si>
+    <t>PRG_Output</t>
+  </si>
+  <si>
+    <t>P_Output</t>
+  </si>
+  <si>
+    <t>FB_ValveControl</t>
+  </si>
+  <si>
+    <t>P_ControlBlock</t>
+  </si>
+  <si>
+    <t>fDeadUp</t>
+  </si>
+  <si>
+    <t>fDeadDown</t>
+  </si>
+  <si>
+    <t>0.23</t>
+  </si>
+  <si>
+    <t>0.215</t>
+  </si>
+  <si>
+    <t>Upper deadband valve?</t>
+  </si>
+  <si>
+    <t>Lower deadband valve?</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>Old</t>
+  </si>
+  <si>
+    <t>Removed control blocks (FF,PF,++)</t>
+  </si>
+  <si>
+    <t>PRG_ManualDriving</t>
+  </si>
+  <si>
+    <t>FB_InitialPosition</t>
+  </si>
+  <si>
+    <t>FB_InitialPos</t>
+  </si>
+  <si>
+    <t>P_Filtering_1</t>
+  </si>
+  <si>
+    <t>Filter constants</t>
+  </si>
+  <si>
+    <t>FB_Filtering</t>
+  </si>
+  <si>
+    <t>FB_Filter</t>
+  </si>
+  <si>
+    <t>DiscreteTransferFcn1_states</t>
+  </si>
+  <si>
+    <t>DiscreteTransferFcn1_icLoad</t>
+  </si>
+  <si>
+    <t>FilterState</t>
+  </si>
+  <si>
+    <t>InitialCondition</t>
+  </si>
+  <si>
+    <t>ssMethodType</t>
+  </si>
+  <si>
+    <t>FilterMode</t>
+  </si>
+  <si>
+    <t>P_Filtering</t>
+  </si>
+  <si>
+    <t>PRG_Filter</t>
+  </si>
+  <si>
+    <t>FB_CylinderScaling</t>
+  </si>
+  <si>
+    <t>FB_PositionInputScaling</t>
+  </si>
+  <si>
+    <t>Curve fitting values</t>
   </si>
 </sst>
 </file>
@@ -89,7 +194,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -108,8 +213,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -117,11 +228,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -133,6 +259,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -469,55 +604,199 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{478C50F6-E11B-4801-A279-E999433C1C1C}">
-  <dimension ref="C4:E7"/>
+  <dimension ref="C4:M16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="1"/>
     <col min="3" max="3" width="27.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="18.6640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.6640625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="6" max="10" width="8.88671875" style="1"/>
+    <col min="11" max="11" width="25.44140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="30.77734375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="28.88671875" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C5" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C6" s="1" t="s">
+      <c r="K6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>9</v>
+      <c r="K7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="K8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C9" s="2"/>
+      <c r="K9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="K13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="K15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Twincat Update: 13.02 (10:21)
</commit_message>
<xml_diff>
--- a/Twincat/Parameters.xlsx
+++ b/Twincat/Parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kimro\Documents\Bachelor\Twincat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689332FD-F6D4-4377-BDE9-85228FBC28F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A3E1E6C-7F31-4A7E-8C96-0C0CEF4B7B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75D9AD79-BFC7-4289-9BE2-FD8EA15511B0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="85">
   <si>
     <t>nOffset</t>
   </si>
@@ -128,9 +128,6 @@
     <t>FB_InitialPos</t>
   </si>
   <si>
-    <t>P_Filtering_1</t>
-  </si>
-  <si>
     <t>Filter constants</t>
   </si>
   <si>
@@ -171,6 +168,129 @@
   </si>
   <si>
     <t>Curve fitting values</t>
+  </si>
+  <si>
+    <t>FB_Normalization</t>
+  </si>
+  <si>
+    <t>FB_Normalize</t>
+  </si>
+  <si>
+    <t>FB_JoystickInputScaling</t>
+  </si>
+  <si>
+    <t>FB_JoystickScaler</t>
+  </si>
+  <si>
+    <t>400 [bar]</t>
+  </si>
+  <si>
+    <t>Max value pressure?</t>
+  </si>
+  <si>
+    <t>Pressure:</t>
+  </si>
+  <si>
+    <t>16090.0</t>
+  </si>
+  <si>
+    <t>Raw signal for piston at max?</t>
+  </si>
+  <si>
+    <t>125.0</t>
+  </si>
+  <si>
+    <t>Raw signal for piston at min?</t>
+  </si>
+  <si>
+    <t>fbNormCylinderPosition:</t>
+  </si>
+  <si>
+    <t>fbNormJoystick:</t>
+  </si>
+  <si>
+    <t>14745.0</t>
+  </si>
+  <si>
+    <t>Raw signal for joystick at max?</t>
+  </si>
+  <si>
+    <t>Raw signal for joystick at min?</t>
+  </si>
+  <si>
+    <t>1620.0</t>
+  </si>
+  <si>
+    <t>8140.0</t>
+  </si>
+  <si>
+    <t>Raw signal for joystick at neutral?</t>
+  </si>
+  <si>
+    <t>100.0</t>
+  </si>
+  <si>
+    <t>Deadband set value</t>
+  </si>
+  <si>
+    <t>fbNormSpoolPosition:</t>
+  </si>
+  <si>
+    <t>8355.0</t>
+  </si>
+  <si>
+    <t>12645.0</t>
+  </si>
+  <si>
+    <t>15.0</t>
+  </si>
+  <si>
+    <t>raw signal spool at neutral position?</t>
+  </si>
+  <si>
+    <t>raw signal spool at max position?</t>
+  </si>
+  <si>
+    <t>raw signal spool at min position?</t>
+  </si>
+  <si>
+    <t>Spool deadband?</t>
+  </si>
+  <si>
+    <t>fbNormFlow:</t>
+  </si>
+  <si>
+    <t>150.0</t>
+  </si>
+  <si>
+    <t>32767.0</t>
+  </si>
+  <si>
+    <t>15270.0</t>
+  </si>
+  <si>
+    <t>25.0</t>
+  </si>
+  <si>
+    <t>Max flow L/min?</t>
+  </si>
+  <si>
+    <t>raw signal max flow?</t>
+  </si>
+  <si>
+    <t>raw signal min flow?</t>
+  </si>
+  <si>
+    <t>Neutral flow?????</t>
+  </si>
+  <si>
+    <t>Deadband flow???</t>
+  </si>
+  <si>
+    <t>PRG_ScaledInputs</t>
+  </si>
+  <si>
+    <t>P_Inputs</t>
   </si>
 </sst>
 </file>
@@ -247,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -267,7 +387,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -604,13 +727,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{478C50F6-E11B-4801-A279-E999433C1C1C}">
-  <dimension ref="C4:M16"/>
+  <dimension ref="C4:M34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="1"/>
     <col min="3" max="3" width="27.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="18.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="22.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="33.44140625" style="1" customWidth="1"/>
     <col min="6" max="10" width="8.88671875" style="1"/>
     <col min="11" max="11" width="25.44140625" style="1" customWidth="1"/>
     <col min="12" max="12" width="30.77734375" style="1" customWidth="1"/>
@@ -722,10 +845,10 @@
         <v>22</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="3:13" x14ac:dyDescent="0.3">
@@ -739,60 +862,229 @@
         <v>23</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="3:13" x14ac:dyDescent="0.3">
       <c r="K13" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="E14" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="3:13" x14ac:dyDescent="0.3">
       <c r="K15" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C16" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="1" t="s">
+    </row>
+    <row r="17" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="K17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>43</v>
+      <c r="L17" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C18" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="8"/>
+      <c r="K18" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C20" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="D21" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C22" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="D23" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="D24" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="D25" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C26" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="D27" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="D28" s="1">
+        <v>4071</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="D29" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="D31" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="32" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="D32" s="1">
+        <v>0</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D33" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D34" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Twincat Update: 13.02 (14:04)
Scriptet funker for manuell kjøring. Verdier blir filtrert og ser bra ut.
</commit_message>
<xml_diff>
--- a/Twincat/Parameters.xlsx
+++ b/Twincat/Parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kimro\Documents\Bachelor\Twincat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A3E1E6C-7F31-4A7E-8C96-0C0CEF4B7B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09485924-6319-453B-9F23-23C00445AEBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75D9AD79-BFC7-4289-9BE2-FD8EA15511B0}"/>
   </bookViews>
@@ -367,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -388,9 +388,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -930,7 +927,6 @@
       <c r="C18" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E18" s="8"/>
       <c r="K18" s="2" t="s">
         <v>47</v>
       </c>

</xml_diff>